<commit_message>
Refactor ParamsManager and integrate SortData for recipe management
- Updated ParamsManager to utilize SortData for storing and loading widget parameters in YAML format instead of Excel.
- Removed the dependency on Excel for parameter management, streamlining the process of saving and loading recipes.
- Introduced SortWidget for managing sorting parameters with enhanced UI features.
- Added SortExcelExporter for optional export/import of recipes to/from Excel.
- Deleted unused SortWidget class to clean up the codebase.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/value_settings.xlsx
+++ b/value_settings.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>40000.0</t>
+          <t>20000.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>16.01140022277832</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"CAP": []}</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{"name": "CAP", "x1": 99, "y1": 45, "x2": 302, "y2": 209}]</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>region</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">

</xml_diff>